<commit_message>
Adición de una columna indicando Pass, Fail y Ongoing
</commit_message>
<xml_diff>
--- a/R/QA_checklist.xlsx
+++ b/R/QA_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\inesg\Desktop\EpiChron\PROYECTO1\QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D948DDB3-7BE9-46D1-AB9D-BF72479E03FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1BC4E96-F8E2-4ECA-8896-FD055B269F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{285F8255-B628-430A-8034-E2848FC9E0E3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{285F8255-B628-430A-8034-E2848FC9E0E3}"/>
   </bookViews>
   <sheets>
     <sheet name="MADRE" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="157">
   <si>
     <t>Check</t>
   </si>
@@ -60,6 +60,9 @@
     <t>Resultado obtenido</t>
   </si>
   <si>
+    <t>Estado</t>
+  </si>
+  <si>
     <t>Estructura de la tabla</t>
   </si>
   <si>
@@ -508,14 +511,28 @@
   </si>
   <si>
     <t>Integridad referencial EMBARAZO -&gt; USO_SERVICIO</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -536,7 +553,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -639,6 +656,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -667,32 +696,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,15 +739,15 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FFFFFF99"/>
       <color rgb="FFFFFF00"/>
       <color rgb="FFFF9966"/>
+      <color rgb="FF66FFFF"/>
       <color rgb="FFFF5050"/>
+      <color rgb="FFFF99CC"/>
+      <color rgb="FFFF6699"/>
+      <color rgb="FFFFFF99"/>
       <color rgb="FFCCFFFF"/>
-      <color rgb="FF66FFFF"/>
-      <color rgb="FFFF99CC"/>
       <color rgb="FFFFCCCC"/>
-      <color rgb="FFFF6699"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1040,154 +1078,184 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77968D7B-81BF-4A61-9BE3-40DAF4F112E9}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.6640625" customWidth="1"/>
     <col min="2" max="2" width="16.88671875" customWidth="1"/>
     <col min="3" max="3" width="39.77734375" customWidth="1"/>
     <col min="4" max="4" width="35.6640625" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="E1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="6" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D2" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="D4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="D5" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="D6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="D7" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="B8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="D8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="D9" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>110</v>
+      <c r="C10" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1197,7 +1265,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA9D0AC8-046B-4403-8143-47181F9112AA}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5546875" customWidth="1"/>
@@ -1206,242 +1274,293 @@
     <col min="4" max="4" width="77.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="E5" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="D6" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="D7" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="B9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="E9" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="B11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="3" t="s">
+      <c r="D11" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="E11" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="D13" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="D14" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="B15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="D15" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="B16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="D16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>123</v>
+      <c r="B17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E17" s="28" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1451,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4B22DCF-7F96-4533-90EA-FB2F1E185759}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.109375" customWidth="1"/>
@@ -1460,186 +1579,225 @@
     <col min="4" max="4" width="78.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="E1" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="9" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="C2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+      <c r="C3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D3" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="D4" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="9" t="s">
+      <c r="B5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="B6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="D6" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="B7" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="9" t="s">
+      <c r="D7" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="B8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="D8" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="B9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="D9" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="B10" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="E10" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="B11" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="E11" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>49</v>
+      <c r="B12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1649,7 +1807,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCDBA703-9E5E-477D-8243-D0A5E84CF2D6}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.5546875" customWidth="1"/>
@@ -1659,106 +1817,127 @@
     <col min="5" max="5" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="E1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="C2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="13" t="s">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="D4" s="14" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="D5" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="D6" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="21"/>
+      <c r="C7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1767,7 +1946,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0DF6C8-3343-4065-ACAF-613DF81890A2}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
@@ -1778,88 +1957,106 @@
     <col min="8" max="8" width="31.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="E1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="16" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="C2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="16" t="s">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+      <c r="C4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
+      <c r="D4" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>139</v>
+      <c r="D6" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1869,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809EF570-AE2B-4960-AC2A-6FEFA188C54B}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.44140625" customWidth="1"/>
@@ -1880,130 +2077,157 @@
     <col min="8" max="8" width="32.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="18" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="19" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="C2" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="19" t="s">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="B4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="19" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="C4" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="D4" s="20" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="19" t="s">
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="19" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="B6" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="D6" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
+      <c r="B7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="19" t="s">
+      <c r="D7" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="19" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="B8" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="D8" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>82</v>
+      <c r="B9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2013,7 +2237,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4A5D912-A48B-4260-9078-DCBDD13D159B}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -2023,130 +2247,157 @@
     <col min="8" max="8" width="32.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="E1" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="C2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="13" t="s">
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="D4" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="D5" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="B6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="D6" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="B7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="D7" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>87</v>
+      <c r="B8" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2156,7 +2407,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25ED159F-3FF4-4385-B1BE-E342CE86CF2C}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="57" customWidth="1"/>
@@ -2167,158 +2418,191 @@
     <col min="8" max="8" width="25.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="23" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="D2" s="24" t="b">
+      <c r="E1" s="33" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="25" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" s="4" t="b">
+      <c r="E2" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A3" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="24" t="b">
+      <c r="E3" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="25" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A5" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" s="4" t="b">
+      <c r="E4" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A5" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="23" t="s">
-        <v>153</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="24" t="b">
+      <c r="E5" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="25" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="E6" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A7" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="4" t="b">
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="24" t="s">
+      <c r="E7" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="D8" s="24" t="b">
+      <c r="B8" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="25" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="E8" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A9" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="D9" s="4" t="b">
+      <c r="B9" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="24" t="s">
+      <c r="E9" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A10" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="24" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
+      <c r="B10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="25" t="s">
         <v>103</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="D10" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="A11" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>104</v>
+      <c r="B11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>